<commit_message>
minor correction in yr0 model
</commit_message>
<xml_diff>
--- a/DRM2/Model_inputs.xlsx
+++ b/DRM2/Model_inputs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jin.tong\Documents\Rprojects\Dental_Reform_Modelling_2\DRM2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B13C6DA-D32D-4856-AB2D-B90528631E39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F29C9CE-7ABF-48BB-ABAE-175C46D7441A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13230" xr2:uid="{2D6CAA86-23AB-4FD8-B2E4-E0C7C9BB22FE}"/>
   </bookViews>
@@ -851,7 +851,7 @@
     <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="112">
+  <cellXfs count="111">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -991,7 +991,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
     <xf numFmtId="8" fontId="10" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="8" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="10" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="8" fontId="10" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1007,7 +1006,6 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="9" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="6" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -1028,7 +1026,6 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="9" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="10" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
@@ -1046,7 +1043,6 @@
     <xf numFmtId="169" fontId="10" fillId="0" borderId="2" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1059,6 +1055,9 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="10" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="10" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="5" builtinId="3"/>
@@ -1416,31 +1415,31 @@
       <c r="B1" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="86" t="s">
+      <c r="C1" s="84" t="s">
         <v>23</v>
       </c>
-      <c r="D1" s="89" t="s">
+      <c r="D1" s="87" t="s">
         <v>107</v>
       </c>
-      <c r="E1" s="90" t="s">
+      <c r="E1" s="88" t="s">
         <v>106</v>
       </c>
-      <c r="F1" s="91" t="s">
+      <c r="F1" s="89" t="s">
         <v>108</v>
       </c>
-      <c r="G1" s="90" t="s">
+      <c r="G1" s="88" t="s">
         <v>109</v>
       </c>
-      <c r="H1" s="90" t="s">
+      <c r="H1" s="88" t="s">
         <v>110</v>
       </c>
-      <c r="I1" s="90" t="s">
+      <c r="I1" s="88" t="s">
         <v>111</v>
       </c>
-      <c r="J1" s="90" t="s">
+      <c r="J1" s="88" t="s">
         <v>112</v>
       </c>
-      <c r="K1" s="92" t="s">
+      <c r="K1" s="90" t="s">
         <v>113</v>
       </c>
       <c r="L1" s="2" t="s">
@@ -1465,11 +1464,11 @@
       <c r="B2" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="87">
+      <c r="C2" s="85">
         <f>HLOOKUP($C$14, D1:K2, 2,FALSE)</f>
-        <v>79906424</v>
-      </c>
-      <c r="D2" s="93">
+        <v>6840730</v>
+      </c>
+      <c r="D2" s="91">
         <v>79906424</v>
       </c>
       <c r="E2" s="59">
@@ -1490,7 +1489,7 @@
       <c r="J2" s="59">
         <v>11300162</v>
       </c>
-      <c r="K2" s="94">
+      <c r="K2" s="92">
         <v>6840730</v>
       </c>
       <c r="L2" t="s">
@@ -1516,33 +1515,33 @@
       <c r="B3" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="88">
+      <c r="C3" s="86">
         <f>HLOOKUP($C$14, $D$1:K3, 3,FALSE)</f>
-        <v>36.699604137603508</v>
-      </c>
-      <c r="D3" s="95">
-        <v>36.699604137603508</v>
+        <v>36.356464583335409</v>
+      </c>
+      <c r="D3" s="93">
+        <v>36.69960414032488</v>
       </c>
       <c r="E3" s="60">
-        <v>35.357614315609389</v>
+        <v>35.357614367301231</v>
       </c>
       <c r="F3" s="60">
-        <v>38.261389118920356</v>
+        <v>38.261389120672945</v>
       </c>
       <c r="G3" s="60">
-        <v>34.59674669069814</v>
+        <v>34.596746702435532</v>
       </c>
       <c r="H3" s="60">
-        <v>38.669432475719425</v>
+        <v>38.669432467987427</v>
       </c>
       <c r="I3" s="60">
-        <v>37.749442845846509</v>
+        <v>37.749442809183094</v>
       </c>
       <c r="J3" s="60">
-        <v>35.839428789649212</v>
-      </c>
-      <c r="K3" s="96">
-        <v>36.356464595445232</v>
+        <v>35.839428805227314</v>
+      </c>
+      <c r="K3" s="94">
+        <v>36.356464583335409</v>
       </c>
       <c r="L3" t="s">
         <v>90</v>
@@ -1564,41 +1563,41 @@
       <c r="B4" s="37" t="s">
         <v>74</v>
       </c>
-      <c r="C4" s="88">
+      <c r="C4" s="86">
         <f>HLOOKUP($C$14, $D$1:K4, 4,FALSE)</f>
-        <v>71196623.783999994</v>
-      </c>
-      <c r="D4" s="106">
+        <v>4978704.9651913978</v>
+      </c>
+      <c r="D4" s="103">
         <f>D2*D5</f>
-        <v>71196623.783999994</v>
-      </c>
-      <c r="E4" s="106">
+        <v>69757023.386649758</v>
+      </c>
+      <c r="E4" s="103">
         <f t="shared" ref="E4:K4" si="0">E2*E5</f>
-        <v>7729465.5474233003</v>
-      </c>
-      <c r="F4" s="106">
+        <v>7693979.2035698527</v>
+      </c>
+      <c r="F4" s="103">
         <f t="shared" si="0"/>
-        <v>11395202.7637231</v>
-      </c>
-      <c r="G4" s="106">
+        <v>11384280.923911804</v>
+      </c>
+      <c r="G4" s="103">
         <f t="shared" si="0"/>
-        <v>13882922.877151363</v>
-      </c>
-      <c r="H4" s="106">
+        <v>13867346.88603784</v>
+      </c>
+      <c r="H4" s="103">
         <f t="shared" si="0"/>
-        <v>11460696.035016203</v>
-      </c>
-      <c r="I4" s="106">
+        <v>11444759.250505202</v>
+      </c>
+      <c r="I4" s="103">
         <f t="shared" si="0"/>
-        <v>10655602.354408357</v>
-      </c>
-      <c r="J4" s="106">
+        <v>10642037.43300893</v>
+      </c>
+      <c r="J4" s="103">
         <f t="shared" si="0"/>
-        <v>9805453.0896568112</v>
-      </c>
-      <c r="K4" s="106">
-        <f t="shared" si="0"/>
-        <v>4987572.5109168328</v>
+        <v>9792739.5667073261</v>
+      </c>
+      <c r="K4" s="103">
+        <f>K2*K5</f>
+        <v>4978704.9651913978</v>
       </c>
       <c r="L4" t="s">
         <v>89</v>
@@ -1620,33 +1619,33 @@
       <c r="B5" s="37" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="88">
+      <c r="C5" s="86">
         <f>HLOOKUP($C$14, $D$1:K5, 5,FALSE)</f>
-        <v>0.89100000000000001</v>
-      </c>
-      <c r="D5" s="107">
-        <v>0.89100000000000001</v>
-      </c>
-      <c r="E5" s="84">
-        <v>0.87693778330688543</v>
-      </c>
-      <c r="F5" s="84">
-        <v>0.96432703092359395</v>
-      </c>
-      <c r="G5" s="84">
-        <v>0.87423887031006231</v>
-      </c>
-      <c r="H5" s="84">
-        <v>0.85576181958681041</v>
-      </c>
-      <c r="I5" s="84">
-        <v>0.89827948564569471</v>
-      </c>
-      <c r="J5" s="84">
-        <v>0.86772677149732991</v>
-      </c>
-      <c r="K5" s="99">
-        <v>0.72909945443203183</v>
+        <v>0.72780316796473443</v>
+      </c>
+      <c r="D5" s="108">
+        <v>0.87298392162624827</v>
+      </c>
+      <c r="E5" s="109">
+        <v>0.87291172024656394</v>
+      </c>
+      <c r="F5" s="109">
+        <v>0.96340276256472102</v>
+      </c>
+      <c r="G5" s="109">
+        <v>0.87325801512592405</v>
+      </c>
+      <c r="H5" s="109">
+        <v>0.85457183150320448</v>
+      </c>
+      <c r="I5" s="109">
+        <v>0.89713594723160772</v>
+      </c>
+      <c r="J5" s="109">
+        <v>0.86660169710021207</v>
+      </c>
+      <c r="K5" s="110">
+        <v>0.72780316796473443</v>
       </c>
       <c r="L5" t="s">
         <v>89</v>
@@ -1662,32 +1661,32 @@
       <c r="B6" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="88" t="str">
+      <c r="C6" s="86" t="str">
         <f>HLOOKUP($C$14, $D$1:K6, 6,FALSE)</f>
         <v>2024/2025</v>
       </c>
-      <c r="D6" s="97" t="s">
+      <c r="D6" s="95" t="s">
         <v>99</v>
       </c>
-      <c r="E6" s="82" t="s">
+      <c r="E6" s="81" t="s">
         <v>99</v>
       </c>
-      <c r="F6" s="82" t="s">
+      <c r="F6" s="81" t="s">
         <v>99</v>
       </c>
-      <c r="G6" s="82" t="s">
+      <c r="G6" s="81" t="s">
         <v>99</v>
       </c>
-      <c r="H6" s="82" t="s">
+      <c r="H6" s="81" t="s">
         <v>99</v>
       </c>
-      <c r="I6" s="82" t="s">
+      <c r="I6" s="81" t="s">
         <v>99</v>
       </c>
-      <c r="J6" s="82" t="s">
+      <c r="J6" s="81" t="s">
         <v>99</v>
       </c>
-      <c r="K6" s="100" t="s">
+      <c r="K6" s="97" t="s">
         <v>99</v>
       </c>
       <c r="L6" t="s">
@@ -1704,32 +1703,32 @@
       <c r="B7" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="C7" s="88">
+      <c r="C7" s="86">
         <f>HLOOKUP($C$14, $D$1:K7, 7,FALSE)</f>
+        <v>0.69145381562128583</v>
+      </c>
+      <c r="D7" s="96">
         <v>0.73000215782769395</v>
       </c>
-      <c r="D7" s="98">
-        <v>0.73000215782769395</v>
-      </c>
-      <c r="E7" s="83">
+      <c r="E7" s="82">
         <v>0.75758755360424745</v>
       </c>
-      <c r="F7" s="83">
+      <c r="F7" s="82">
         <v>0.83008638928067702</v>
       </c>
-      <c r="G7" s="83">
+      <c r="G7" s="82">
         <v>0.76568397546477152</v>
       </c>
-      <c r="H7" s="83">
+      <c r="H7" s="82">
         <v>0.61631321718089616</v>
       </c>
-      <c r="I7" s="83">
+      <c r="I7" s="82">
         <v>0.47847479498813639</v>
       </c>
-      <c r="J7" s="83">
+      <c r="J7" s="82">
         <v>0.751447645420808</v>
       </c>
-      <c r="K7" s="101">
+      <c r="K7" s="98">
         <v>0.69145381562128583</v>
       </c>
       <c r="L7" t="s">
@@ -1746,33 +1745,33 @@
       <c r="B8" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="C8" s="88">
+      <c r="C8" s="86">
         <f>HLOOKUP($C$14, $D$1:K8, 8,FALSE)</f>
+        <v>6634186.231741244</v>
+      </c>
+      <c r="D8" s="95">
         <v>77493790.564527199</v>
       </c>
-      <c r="D8" s="97">
-        <v>77493790.564527199</v>
-      </c>
-      <c r="E8" s="85">
-        <v>8548027</v>
-      </c>
-      <c r="F8" s="85">
-        <v>11459955</v>
-      </c>
-      <c r="G8" s="85">
-        <v>15400542</v>
-      </c>
-      <c r="H8" s="85">
-        <v>12988030</v>
-      </c>
-      <c r="I8" s="85">
-        <v>11504076</v>
-      </c>
-      <c r="J8" s="85">
-        <v>10958974</v>
-      </c>
-      <c r="K8" s="102">
-        <v>6634186</v>
+      <c r="E8" s="83">
+        <v>8548027.1470198724</v>
+      </c>
+      <c r="F8" s="83">
+        <v>11459955.362403173</v>
+      </c>
+      <c r="G8" s="83">
+        <v>15400542.09654518</v>
+      </c>
+      <c r="H8" s="83">
+        <v>12988030.421915369</v>
+      </c>
+      <c r="I8" s="83">
+        <v>11504075.751371434</v>
+      </c>
+      <c r="J8" s="83">
+        <v>10958973.553530926</v>
+      </c>
+      <c r="K8" s="99">
+        <v>6634186.231741244</v>
       </c>
       <c r="L8" t="s">
         <v>92</v>
@@ -1788,32 +1787,32 @@
       <c r="B9" s="38" t="s">
         <v>77</v>
       </c>
-      <c r="C9" s="88">
+      <c r="C9" s="86">
         <f>HLOOKUP($C$14, $D$1:K9, 9,FALSE)</f>
         <v>1.0434558691517315</v>
       </c>
-      <c r="D9" s="97">
+      <c r="D9" s="95">
         <v>1.0434558691517315</v>
       </c>
-      <c r="E9" s="82">
+      <c r="E9" s="81">
         <v>1.0434558691517315</v>
       </c>
-      <c r="F9" s="82">
+      <c r="F9" s="81">
         <v>1.0434558691517315</v>
       </c>
-      <c r="G9" s="82">
+      <c r="G9" s="81">
         <v>1.0434558691517315</v>
       </c>
-      <c r="H9" s="82">
+      <c r="H9" s="81">
         <v>1.0434558691517315</v>
       </c>
-      <c r="I9" s="82">
+      <c r="I9" s="81">
         <v>1.0434558691517315</v>
       </c>
-      <c r="J9" s="82">
+      <c r="J9" s="81">
         <v>1.0434558691517315</v>
       </c>
-      <c r="K9" s="100">
+      <c r="K9" s="97">
         <v>1.0434558691517315</v>
       </c>
       <c r="L9" t="s">
@@ -1830,32 +1829,32 @@
       <c r="B10" s="37" t="s">
         <v>76</v>
       </c>
-      <c r="C10" s="88">
+      <c r="C10" s="86">
         <f>HLOOKUP($C$14, $D$1:K10, 10,FALSE)</f>
         <v>10</v>
       </c>
-      <c r="D10" s="97">
+      <c r="D10" s="95">
         <v>10</v>
       </c>
-      <c r="E10" s="82">
+      <c r="E10" s="81">
         <v>10</v>
       </c>
-      <c r="F10" s="82">
+      <c r="F10" s="81">
         <v>10</v>
       </c>
-      <c r="G10" s="82">
+      <c r="G10" s="81">
         <v>10</v>
       </c>
-      <c r="H10" s="82">
+      <c r="H10" s="81">
         <v>10</v>
       </c>
-      <c r="I10" s="82">
+      <c r="I10" s="81">
         <v>10</v>
       </c>
-      <c r="J10" s="82">
+      <c r="J10" s="81">
         <v>10</v>
       </c>
-      <c r="K10" s="100">
+      <c r="K10" s="97">
         <v>10</v>
       </c>
       <c r="L10" t="s">
@@ -1869,32 +1868,32 @@
       <c r="B11" s="37" t="s">
         <v>78</v>
       </c>
-      <c r="C11" s="88">
+      <c r="C11" s="86">
         <f>HLOOKUP($C$14, $D$1:K11, 11,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="D11" s="103">
+      <c r="D11" s="100">
         <v>0</v>
       </c>
-      <c r="E11" s="104">
+      <c r="E11" s="101">
         <v>0</v>
       </c>
-      <c r="F11" s="104">
+      <c r="F11" s="101">
         <v>0</v>
       </c>
-      <c r="G11" s="104">
+      <c r="G11" s="101">
         <v>0</v>
       </c>
-      <c r="H11" s="104">
+      <c r="H11" s="101">
         <v>0</v>
       </c>
-      <c r="I11" s="104">
+      <c r="I11" s="101">
         <v>0</v>
       </c>
-      <c r="J11" s="104">
+      <c r="J11" s="101">
         <v>0</v>
       </c>
-      <c r="K11" s="105">
+      <c r="K11" s="102">
         <v>0</v>
       </c>
       <c r="L11" t="s">
@@ -1910,7 +1909,7 @@
         <v>88</v>
       </c>
       <c r="C13" s="40" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D13" s="32"/>
       <c r="E13" s="24"/>
@@ -1928,7 +1927,7 @@
         <v>105</v>
       </c>
       <c r="C14" s="42" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="D14" s="32"/>
       <c r="E14" s="24"/>
@@ -1974,31 +1973,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="57.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="109" t="s">
+      <c r="A1" s="105" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="109"/>
-      <c r="C1" s="109"/>
-      <c r="D1" s="111" t="s">
+      <c r="B1" s="105"/>
+      <c r="C1" s="105"/>
+      <c r="D1" s="107" t="s">
         <v>57</v>
       </c>
-      <c r="E1" s="111"/>
-      <c r="F1" s="111"/>
-      <c r="G1" s="111"/>
+      <c r="E1" s="107"/>
+      <c r="F1" s="107"/>
+      <c r="G1" s="107"/>
     </row>
     <row r="2" spans="1:25" ht="57.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="110" t="s">
+      <c r="B2" s="106" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="110"/>
-      <c r="D2" s="108" t="s">
+      <c r="C2" s="106"/>
+      <c r="D2" s="104" t="s">
         <v>35</v>
       </c>
-      <c r="E2" s="108"/>
-      <c r="F2" s="108"/>
+      <c r="E2" s="104"/>
+      <c r="F2" s="104"/>
       <c r="G2" s="44" t="s">
         <v>58</v>
       </c>
@@ -2062,10 +2061,10 @@
         <v>1454518</v>
       </c>
       <c r="E4" s="60">
-        <v>36.699604137603508</v>
+        <v>36.69960414032488</v>
       </c>
       <c r="F4" s="60">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G4" s="20" t="s">
         <v>38</v>
@@ -2088,10 +2087,10 @@
         <v>1048743</v>
       </c>
       <c r="E5" s="60">
-        <v>179.30876935945406</v>
+        <v>179.30876937275028</v>
       </c>
       <c r="F5" s="60">
-        <v>61.79</v>
+        <v>61.789499318531895</v>
       </c>
       <c r="G5" s="20" t="s">
         <v>38</v>
@@ -2114,10 +2113,10 @@
         <v>387887</v>
       </c>
       <c r="E6" s="60">
-        <v>383.73474400294782</v>
+        <v>383.73474403140273</v>
       </c>
       <c r="F6" s="60">
-        <v>76.02</v>
+        <v>76.024503939645342</v>
       </c>
       <c r="G6" s="20" t="s">
         <v>38</v>
@@ -2140,10 +2139,10 @@
         <v>5383909.7867940795</v>
       </c>
       <c r="E7" s="60">
-        <v>179.30876935945406</v>
+        <v>179.30876937275028</v>
       </c>
       <c r="F7" s="60">
-        <v>61.79</v>
+        <v>61.789499318531895</v>
       </c>
       <c r="G7" s="20" t="s">
         <v>38</v>
@@ -2166,10 +2165,10 @@
         <v>288474.67457258003</v>
       </c>
       <c r="E8" s="60">
-        <v>110.09881241281053</v>
+        <v>102.75889159290968</v>
       </c>
       <c r="F8" s="60">
-        <v>45.96</v>
+        <v>43.715100994013127</v>
       </c>
       <c r="G8" s="20" t="s">
         <v>38</v>
@@ -2189,13 +2188,13 @@
         <v>13</v>
       </c>
       <c r="D9" s="59">
-        <v>10839611.202428667</v>
+        <v>10810763.73497141</v>
       </c>
       <c r="E9" s="60">
-        <v>36.699604137603508</v>
+        <v>36.69960414032488</v>
       </c>
       <c r="F9" s="60">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G9" s="20" t="s">
         <v>38</v>
@@ -2218,7 +2217,7 @@
         <v>8239111.7975713331</v>
       </c>
       <c r="E10" s="60">
-        <v>36.699604137603508</v>
+        <v>36.69960414032488</v>
       </c>
       <c r="F10" s="57">
         <v>0</v>
@@ -2244,7 +2243,7 @@
         <v>2427992.5386333391</v>
       </c>
       <c r="E11" s="60">
-        <v>143.06520141235922</v>
+        <v>143.06520142296787</v>
       </c>
       <c r="F11" s="57">
         <v>0</v>
@@ -2270,10 +2269,10 @@
         <v>2912626</v>
       </c>
       <c r="E12" s="65">
-        <v>44.039524965124208</v>
+        <v>44.039524968389856</v>
       </c>
       <c r="F12" s="65">
-        <v>17.989999999999998</v>
+        <v>17.987644010001613</v>
       </c>
       <c r="G12" s="66" t="s">
         <v>38</v>
@@ -2306,10 +2305,10 @@
         <v>1454518</v>
       </c>
       <c r="E14" s="69">
-        <v>36.699604137603508</v>
+        <v>36.69960414032488</v>
       </c>
       <c r="F14" s="69">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G14" s="70" t="s">
         <v>39</v>
@@ -2334,10 +2333,10 @@
         <v>1048743</v>
       </c>
       <c r="E15" s="60">
-        <v>179.30876935945406</v>
+        <v>179.30876937275028</v>
       </c>
       <c r="F15" s="60">
-        <v>61.79</v>
+        <v>61.789499318531895</v>
       </c>
       <c r="G15" s="21" t="s">
         <v>39</v>
@@ -2362,10 +2361,10 @@
         <v>387887</v>
       </c>
       <c r="E16" s="60">
-        <v>527.6</v>
+        <v>549.96635307824874</v>
       </c>
       <c r="F16" s="60">
-        <v>76.02</v>
+        <v>70.007057148052098</v>
       </c>
       <c r="G16" s="21" t="s">
         <v>39</v>
@@ -2390,10 +2389,10 @@
         <v>5383909.7867940795</v>
       </c>
       <c r="E17" s="60">
-        <v>179.30876935945406</v>
+        <v>179.30876937275028</v>
       </c>
       <c r="F17" s="60">
-        <v>61.79</v>
+        <v>61.789499318531895</v>
       </c>
       <c r="G17" s="21" t="s">
         <v>39</v>
@@ -2418,10 +2417,10 @@
         <v>288474.67457258003</v>
       </c>
       <c r="E18" s="60">
-        <v>256.89722896322456</v>
+        <v>248.09003281726135</v>
       </c>
       <c r="F18" s="60">
-        <v>45.96</v>
+        <v>45.962687596827379</v>
       </c>
       <c r="G18" s="21" t="s">
         <v>39</v>
@@ -2443,13 +2442,13 @@
         <v>Returning band 1</v>
       </c>
       <c r="D19" s="59">
-        <v>10839611.202428667</v>
+        <v>10810763.73497141</v>
       </c>
       <c r="E19" s="60">
-        <v>36.699604137603508</v>
+        <v>35.441433259608765</v>
       </c>
       <c r="F19" s="60">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G19" s="21" t="s">
         <v>39</v>
@@ -2474,7 +2473,7 @@
         <v>8239111.7975713331</v>
       </c>
       <c r="E20" s="60">
-        <v>36.699604137603508</v>
+        <v>35.441433259608765</v>
       </c>
       <c r="F20" s="57">
         <v>0</v>
@@ -2502,7 +2501,7 @@
         <v>2427992.5386333391</v>
       </c>
       <c r="E21" s="60">
-        <v>143.06520141235922</v>
+        <v>143.06520142296787</v>
       </c>
       <c r="F21" s="57">
         <v>0</v>
@@ -2533,7 +2532,7 @@
         <v>75</v>
       </c>
       <c r="F22" s="65">
-        <v>17.989999999999998</v>
+        <v>17.987644010001613</v>
       </c>
       <c r="G22" s="50" t="s">
         <v>39</v>
@@ -2561,10 +2560,10 @@
         <v>194103</v>
       </c>
       <c r="E24" s="69">
-        <v>35.357614315609389</v>
+        <v>35.357614367301231</v>
       </c>
       <c r="F24" s="69">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G24" s="52" t="s">
         <v>38</v>
@@ -2587,10 +2586,10 @@
         <v>118717</v>
       </c>
       <c r="E25" s="60">
-        <v>172.12694195717168</v>
+        <v>172.12694220881644</v>
       </c>
       <c r="F25" s="60">
-        <v>61.79</v>
+        <v>61.789499318531895</v>
       </c>
       <c r="G25" s="20" t="s">
         <v>38</v>
@@ -2613,10 +2612,10 @@
         <v>37987</v>
       </c>
       <c r="E26" s="60">
-        <v>367.70057324312836</v>
+        <v>367.70057378069635</v>
       </c>
       <c r="F26" s="60">
-        <v>93.01</v>
+        <v>76.024503939645342</v>
       </c>
       <c r="G26" s="20" t="s">
         <v>38</v>
@@ -2639,10 +2638,10 @@
         <v>554643.05690516951</v>
       </c>
       <c r="E27" s="60">
-        <v>172.12694195717168</v>
+        <v>172.12694220881644</v>
       </c>
       <c r="F27" s="60">
-        <v>61.79</v>
+        <v>61.789499318531895</v>
       </c>
       <c r="G27" s="20" t="s">
         <v>38</v>
@@ -2665,10 +2664,10 @@
         <v>33194.381980936079</v>
       </c>
       <c r="E28" s="60">
-        <v>106.07284294682816</v>
+        <v>99.001320228443461</v>
       </c>
       <c r="F28" s="60">
-        <v>45.96</v>
+        <v>43.715100994013127</v>
       </c>
       <c r="G28" s="20" t="s">
         <v>38</v>
@@ -2688,13 +2687,13 @@
         <v>13</v>
       </c>
       <c r="D29" s="59">
-        <v>1341014.7366673516</v>
+        <v>1312167.2692100937</v>
       </c>
       <c r="E29" s="60">
-        <v>35.357614315609389</v>
+        <v>35.357614367301231</v>
       </c>
       <c r="F29" s="60">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G29" s="20" t="s">
         <v>38</v>
@@ -2717,7 +2716,7 @@
         <v>1028784.2633326487</v>
       </c>
       <c r="E30" s="60">
-        <v>35.357614315609389</v>
+        <v>35.357614367301231</v>
       </c>
       <c r="F30" s="71">
         <v>0</v>
@@ -2743,7 +2742,7 @@
         <v>254288.56111389436</v>
       </c>
       <c r="E31" s="60">
-        <v>137.33503223275483</v>
+        <v>137.33503243353479</v>
       </c>
       <c r="F31" s="71">
         <v>0</v>
@@ -2769,10 +2768,10 @@
         <v>337669</v>
       </c>
       <c r="E32" s="65">
-        <v>42.429137178731267</v>
+        <v>42.429137240761477</v>
       </c>
       <c r="F32" s="65">
-        <v>17.989999999999998</v>
+        <v>17.987644010001613</v>
       </c>
       <c r="G32" s="66" t="s">
         <v>38</v>
@@ -2805,10 +2804,10 @@
         <v>194103</v>
       </c>
       <c r="E34" s="69">
-        <v>35.357614315609389</v>
+        <v>35.357614367301231</v>
       </c>
       <c r="F34" s="75">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G34" s="70" t="s">
         <v>39</v>
@@ -2833,10 +2832,10 @@
         <v>118717</v>
       </c>
       <c r="E35" s="60">
-        <v>172.12694195717168</v>
-      </c>
-      <c r="F35" s="76">
-        <v>61.79</v>
+        <v>172.12694220881644</v>
+      </c>
+      <c r="F35" s="60">
+        <v>61.789499318531895</v>
       </c>
       <c r="G35" s="21" t="s">
         <v>39</v>
@@ -2861,10 +2860,10 @@
         <v>37987</v>
       </c>
       <c r="E36" s="60">
-        <v>527.6</v>
-      </c>
-      <c r="F36" s="76">
-        <v>76.02</v>
+        <v>549.96635307824874</v>
+      </c>
+      <c r="F36" s="60">
+        <v>70.007057148052098</v>
       </c>
       <c r="G36" s="21" t="s">
         <v>39</v>
@@ -2889,10 +2888,10 @@
         <v>554643.05690516951</v>
       </c>
       <c r="E37" s="60">
-        <v>172.12694195717168</v>
-      </c>
-      <c r="F37" s="76">
-        <v>61.79</v>
+        <v>172.12694220881644</v>
+      </c>
+      <c r="F37" s="60">
+        <v>61.789499318531895</v>
       </c>
       <c r="G37" s="21" t="s">
         <v>39</v>
@@ -2917,10 +2916,10 @@
         <v>33194.381980936079</v>
       </c>
       <c r="E38" s="60">
-        <v>256.89722896322456</v>
-      </c>
-      <c r="F38" s="76">
-        <v>45.96</v>
+        <v>248.09003281726135</v>
+      </c>
+      <c r="F38" s="60">
+        <v>45.962687596827379</v>
       </c>
       <c r="G38" s="21" t="s">
         <v>39</v>
@@ -2942,13 +2941,13 @@
         <v>Returning band 1</v>
       </c>
       <c r="D39" s="59">
-        <v>1341014.7366673516</v>
+        <v>1312167.2692100937</v>
       </c>
       <c r="E39" s="60">
-        <v>36.699604137603508</v>
-      </c>
-      <c r="F39" s="76">
-        <v>23.49</v>
+        <v>35.441433259608765</v>
+      </c>
+      <c r="F39" s="60">
+        <v>23.486821568684874</v>
       </c>
       <c r="G39" s="21" t="s">
         <v>39</v>
@@ -2973,7 +2972,7 @@
         <v>1028784.2633326487</v>
       </c>
       <c r="E40" s="60">
-        <v>36.699604137603508</v>
+        <v>35.441433259608765</v>
       </c>
       <c r="F40" s="57">
         <v>0</v>
@@ -3001,7 +3000,7 @@
         <v>254288.56111389436</v>
       </c>
       <c r="E41" s="60">
-        <v>137.33503223275483</v>
+        <v>137.33503243353479</v>
       </c>
       <c r="F41" s="57">
         <v>0</v>
@@ -3025,14 +3024,14 @@
         <f>C32</f>
         <v>Urgent care patients</v>
       </c>
-      <c r="D42" s="77">
+      <c r="D42" s="76">
         <v>414883.17366894055</v>
       </c>
       <c r="E42" s="65">
         <v>75</v>
       </c>
-      <c r="F42" s="78">
-        <v>17.989999999999998</v>
+      <c r="F42" s="77">
+        <v>17.987644010001613</v>
       </c>
       <c r="G42" s="50" t="s">
         <v>39</v>
@@ -3060,10 +3059,10 @@
         <v>311147</v>
       </c>
       <c r="E44" s="69">
-        <v>38.261389118920356</v>
+        <v>38.261389120672945</v>
       </c>
       <c r="F44" s="69">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G44" s="52" t="s">
         <v>38</v>
@@ -3086,10 +3085,10 @@
         <v>282495</v>
       </c>
       <c r="E45" s="60">
-        <v>207.66285073088017</v>
+        <v>207.66285074039229</v>
       </c>
       <c r="F45" s="60">
-        <v>61.79</v>
+        <v>61.789499318531895</v>
       </c>
       <c r="G45" s="20" t="s">
         <v>38</v>
@@ -3112,10 +3111,10 @@
         <v>57825</v>
       </c>
       <c r="E46" s="60">
-        <v>421.90643549709824</v>
+        <v>421.90643551642398</v>
       </c>
       <c r="F46" s="60">
-        <v>60.17</v>
+        <v>76.024503939645342</v>
       </c>
       <c r="G46" s="20" t="s">
         <v>38</v>
@@ -3138,10 +3137,10 @@
         <v>812959.63821323367</v>
       </c>
       <c r="E47" s="60">
-        <v>207.66285073088017</v>
+        <v>207.66285074039229</v>
       </c>
       <c r="F47" s="60">
-        <v>61.79</v>
+        <v>61.789499318531895</v>
       </c>
       <c r="G47" s="20" t="s">
         <v>38</v>
@@ -3164,10 +3163,10 @@
         <v>38012.008066009366</v>
       </c>
       <c r="E48" s="60">
-        <v>114.78416735676106</v>
+        <v>107.13188953788426</v>
       </c>
       <c r="F48" s="60">
-        <v>45.96</v>
+        <v>43.715100994013127</v>
       </c>
       <c r="G48" s="20" t="s">
         <v>38</v>
@@ -3187,13 +3186,13 @@
         <v>13</v>
       </c>
       <c r="D49" s="59">
-        <v>1095285.3521748993</v>
+        <v>1091965.9139768058</v>
       </c>
       <c r="E49" s="60">
-        <v>38.261389118920356</v>
+        <v>38.261389120672945</v>
       </c>
       <c r="F49" s="60">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G49" s="20" t="s">
         <v>38</v>
@@ -3216,7 +3215,7 @@
         <v>942543.64782510081</v>
       </c>
       <c r="E50" s="60">
-        <v>38.261389118920356</v>
+        <v>38.261389120672945</v>
       </c>
       <c r="F50" s="71">
         <v>0</v>
@@ -3242,7 +3241,7 @@
         <v>406870.35372075689</v>
       </c>
       <c r="E51" s="60">
-        <v>165.68809028029631</v>
+        <v>165.68809028788576</v>
       </c>
       <c r="F51" s="71">
         <v>0</v>
@@ -3268,10 +3267,10 @@
         <v>489233</v>
       </c>
       <c r="E52" s="65">
-        <v>45.913666942704424</v>
+        <v>45.913666944807531</v>
       </c>
       <c r="F52" s="65">
-        <v>17.989999999999998</v>
+        <v>17.987644010001613</v>
       </c>
       <c r="G52" s="66" t="s">
         <v>38</v>
@@ -3304,10 +3303,10 @@
         <v>311147</v>
       </c>
       <c r="E54" s="69">
-        <v>38.261389118920356</v>
+        <v>38.261389120672945</v>
       </c>
       <c r="F54" s="69">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G54" s="70" t="s">
         <v>39</v>
@@ -3332,10 +3331,10 @@
         <v>282495</v>
       </c>
       <c r="E55" s="60">
-        <v>207.66285073088017</v>
+        <v>207.66285074039229</v>
       </c>
       <c r="F55" s="60">
-        <v>61.79</v>
+        <v>61.789499318531895</v>
       </c>
       <c r="G55" s="21" t="s">
         <v>39</v>
@@ -3360,10 +3359,10 @@
         <v>57825</v>
       </c>
       <c r="E56" s="60">
-        <v>527.6</v>
+        <v>549.96635307824874</v>
       </c>
       <c r="F56" s="60">
-        <v>76.02</v>
+        <v>70.007057148052098</v>
       </c>
       <c r="G56" s="21" t="s">
         <v>39</v>
@@ -3388,10 +3387,10 @@
         <v>812959.63821323367</v>
       </c>
       <c r="E57" s="60">
-        <v>207.66285073088017</v>
+        <v>207.66285074039229</v>
       </c>
       <c r="F57" s="60">
-        <v>61.79</v>
+        <v>61.789499318531895</v>
       </c>
       <c r="G57" s="21" t="s">
         <v>39</v>
@@ -3416,10 +3415,10 @@
         <v>38012.008066009366</v>
       </c>
       <c r="E58" s="60">
-        <v>256.89722896322456</v>
+        <v>248.09003281726135</v>
       </c>
       <c r="F58" s="60">
-        <v>45.96</v>
+        <v>45.962687596827379</v>
       </c>
       <c r="G58" s="21" t="s">
         <v>39</v>
@@ -3441,13 +3440,13 @@
         <v>Returning band 1</v>
       </c>
       <c r="D59" s="59">
-        <v>1095285.3521748993</v>
+        <v>1091965.9139768058</v>
       </c>
       <c r="E59" s="60">
-        <v>36.699604137603508</v>
+        <v>35.441433259608765</v>
       </c>
       <c r="F59" s="60">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G59" s="21" t="s">
         <v>39</v>
@@ -3472,7 +3471,7 @@
         <v>942543.64782510081</v>
       </c>
       <c r="E60" s="60">
-        <v>36.699604137603508</v>
+        <v>35.441433259608765</v>
       </c>
       <c r="F60" s="71">
         <v>0</v>
@@ -3500,7 +3499,7 @@
         <v>406870.35372075689</v>
       </c>
       <c r="E61" s="60">
-        <v>165.68809028029631</v>
+        <v>165.68809028788576</v>
       </c>
       <c r="F61" s="71">
         <v>0</v>
@@ -3531,7 +3530,7 @@
         <v>75</v>
       </c>
       <c r="F62" s="65">
-        <v>17.989999999999998</v>
+        <v>17.987644010001613</v>
       </c>
       <c r="G62" s="50" t="s">
         <v>39</v>
@@ -3559,15 +3558,15 @@
         <v>322784</v>
       </c>
       <c r="E64" s="69">
-        <v>34.59674669069814</v>
+        <v>34.596746702435532</v>
       </c>
       <c r="F64" s="69">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G64" s="52" t="s">
         <v>38</v>
       </c>
-      <c r="H64" s="79" t="s">
+      <c r="H64" s="78" t="s">
         <v>109</v>
       </c>
     </row>
@@ -3585,15 +3584,15 @@
         <v>266762</v>
       </c>
       <c r="E65" s="60">
-        <v>166.8656011300537</v>
+        <v>166.865601186665</v>
       </c>
       <c r="F65" s="60">
-        <v>61.79</v>
+        <v>61.789499318531895</v>
       </c>
       <c r="G65" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H65" s="80" t="s">
+      <c r="H65" s="79" t="s">
         <v>109</v>
       </c>
     </row>
@@ -3611,15 +3610,15 @@
         <v>81635</v>
       </c>
       <c r="E66" s="60">
-        <v>359.58714679609233</v>
+        <v>359.58714691808689</v>
       </c>
       <c r="F66" s="60">
-        <v>77.099999999999994</v>
+        <v>76.024503939645342</v>
       </c>
       <c r="G66" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H66" s="80" t="s">
+      <c r="H66" s="79" t="s">
         <v>109</v>
       </c>
     </row>
@@ -3637,15 +3636,15 @@
         <v>1011290.5843589403</v>
       </c>
       <c r="E67" s="60">
-        <v>166.8656011300537</v>
+        <v>166.865601186665</v>
       </c>
       <c r="F67" s="60">
-        <v>61.79</v>
+        <v>61.789499318531895</v>
       </c>
       <c r="G67" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H67" s="80" t="s">
+      <c r="H67" s="79" t="s">
         <v>109</v>
       </c>
     </row>
@@ -3663,15 +3662,15 @@
         <v>58873.951534574953</v>
       </c>
       <c r="E68" s="60">
-        <v>103.79024007209442</v>
+        <v>96.8708907668195</v>
       </c>
       <c r="F68" s="60">
-        <v>45.96</v>
+        <v>43.715100994013127</v>
       </c>
       <c r="G68" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H68" s="80" t="s">
+      <c r="H68" s="79" t="s">
         <v>109</v>
       </c>
     </row>
@@ -3686,18 +3685,18 @@
         <v>13</v>
       </c>
       <c r="D69" s="59">
-        <v>2203513.4425999173</v>
+        <v>2199712.2417933163</v>
       </c>
       <c r="E69" s="60">
-        <v>34.59674669069814</v>
+        <v>34.596746702435532</v>
       </c>
       <c r="F69" s="60">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G69" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H69" s="80" t="s">
+      <c r="H69" s="79" t="s">
         <v>109</v>
       </c>
     </row>
@@ -3715,7 +3714,7 @@
         <v>1693039.5574000832</v>
       </c>
       <c r="E70" s="60">
-        <v>34.59674669069814</v>
+        <v>34.596746702435532</v>
       </c>
       <c r="F70" s="71">
         <v>0</v>
@@ -3723,7 +3722,7 @@
       <c r="G70" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H70" s="80" t="s">
+      <c r="H70" s="79" t="s">
         <v>109</v>
       </c>
     </row>
@@ -3741,7 +3740,7 @@
         <v>484491.46410648461</v>
       </c>
       <c r="E71" s="60">
-        <v>133.13716289362753</v>
+        <v>133.13716293879602</v>
       </c>
       <c r="F71" s="71">
         <v>0</v>
@@ -3749,7 +3748,7 @@
       <c r="G71" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H71" s="80" t="s">
+      <c r="H71" s="79" t="s">
         <v>109</v>
       </c>
     </row>
@@ -3767,15 +3766,15 @@
         <v>508149</v>
       </c>
       <c r="E72" s="65">
-        <v>41.516096028837765</v>
+        <v>41.516096042922634</v>
       </c>
       <c r="F72" s="65">
-        <v>17.989999999999998</v>
+        <v>17.987644010001613</v>
       </c>
       <c r="G72" s="66" t="s">
         <v>38</v>
       </c>
-      <c r="H72" s="81" t="s">
+      <c r="H72" s="80" t="s">
         <v>109</v>
       </c>
     </row>
@@ -3803,10 +3802,10 @@
         <v>322784</v>
       </c>
       <c r="E74" s="69">
-        <v>34.59674669069814</v>
+        <v>34.596746702435532</v>
       </c>
       <c r="F74" s="75">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G74" s="70" t="s">
         <v>39</v>
@@ -3831,10 +3830,10 @@
         <v>266762</v>
       </c>
       <c r="E75" s="60">
-        <v>166.8656011300537</v>
-      </c>
-      <c r="F75" s="76">
-        <v>61.79</v>
+        <v>166.865601186665</v>
+      </c>
+      <c r="F75" s="60">
+        <v>61.789499318531895</v>
       </c>
       <c r="G75" s="21" t="s">
         <v>39</v>
@@ -3859,10 +3858,10 @@
         <v>81635</v>
       </c>
       <c r="E76" s="60">
-        <v>527.6</v>
-      </c>
-      <c r="F76" s="76">
-        <v>76.02</v>
+        <v>549.96635307824874</v>
+      </c>
+      <c r="F76" s="60">
+        <v>70.007057148052098</v>
       </c>
       <c r="G76" s="21" t="s">
         <v>39</v>
@@ -3887,10 +3886,10 @@
         <v>1011290.5843589403</v>
       </c>
       <c r="E77" s="60">
-        <v>166.8656011300537</v>
-      </c>
-      <c r="F77" s="76">
-        <v>61.79</v>
+        <v>166.865601186665</v>
+      </c>
+      <c r="F77" s="60">
+        <v>61.789499318531895</v>
       </c>
       <c r="G77" s="21" t="s">
         <v>39</v>
@@ -3915,10 +3914,10 @@
         <v>58873.951534574953</v>
       </c>
       <c r="E78" s="60">
-        <v>256.89722896322456</v>
-      </c>
-      <c r="F78" s="76">
-        <v>45.96</v>
+        <v>248.09003281726135</v>
+      </c>
+      <c r="F78" s="60">
+        <v>45.962687596827379</v>
       </c>
       <c r="G78" s="21" t="s">
         <v>39</v>
@@ -3940,13 +3939,13 @@
         <v>Returning band 1</v>
       </c>
       <c r="D79" s="59">
-        <v>2203513.4425999173</v>
+        <v>2199712.2417933163</v>
       </c>
       <c r="E79" s="60">
-        <v>36.699604137603508</v>
-      </c>
-      <c r="F79" s="76">
-        <v>23.49</v>
+        <v>35.441433259608765</v>
+      </c>
+      <c r="F79" s="60">
+        <v>23.486821568684874</v>
       </c>
       <c r="G79" s="21" t="s">
         <v>39</v>
@@ -3971,7 +3970,7 @@
         <v>1693039.5574000832</v>
       </c>
       <c r="E80" s="60">
-        <v>36.699604137603508</v>
+        <v>35.441433259608765</v>
       </c>
       <c r="F80" s="57">
         <v>0</v>
@@ -3999,7 +3998,7 @@
         <v>484491.46410648461</v>
       </c>
       <c r="E81" s="60">
-        <v>133.13716289362753</v>
+        <v>133.13716293879602</v>
       </c>
       <c r="F81" s="57">
         <v>0</v>
@@ -4023,14 +4022,14 @@
         <f>C72</f>
         <v>Urgent care patients</v>
       </c>
-      <c r="D82" s="77">
+      <c r="D82" s="76">
         <v>647261.8165114735</v>
       </c>
       <c r="E82" s="65">
         <v>75</v>
       </c>
-      <c r="F82" s="78">
-        <v>17.989999999999998</v>
+      <c r="F82" s="77">
+        <v>17.987644010001613</v>
       </c>
       <c r="G82" s="50" t="s">
         <v>39</v>
@@ -4058,15 +4057,15 @@
         <v>170846</v>
       </c>
       <c r="E84" s="69">
-        <v>38.669432475719425</v>
+        <v>38.669432467987427</v>
       </c>
       <c r="F84" s="69">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G84" s="52" t="s">
         <v>38</v>
       </c>
-      <c r="H84" s="79" t="s">
+      <c r="H84" s="78" t="s">
         <v>110</v>
       </c>
     </row>
@@ -4084,15 +4083,15 @@
         <v>115637</v>
       </c>
       <c r="E85" s="60">
-        <v>178.32811346650587</v>
+        <v>178.32811343084896</v>
       </c>
       <c r="F85" s="60">
-        <v>61.79</v>
+        <v>61.789499318531895</v>
       </c>
       <c r="G85" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H85" s="80" t="s">
+      <c r="H85" s="79" t="s">
         <v>110</v>
       </c>
     </row>
@@ -4110,15 +4109,15 @@
         <v>71990</v>
       </c>
       <c r="E86" s="60">
-        <v>397.14038931119291</v>
+        <v>397.14038923178424</v>
       </c>
       <c r="F86" s="60">
-        <v>63.58</v>
+        <v>76.024503939645342</v>
       </c>
       <c r="G86" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H86" s="80" t="s">
+      <c r="H86" s="79" t="s">
         <v>110</v>
       </c>
     </row>
@@ -4136,15 +4135,15 @@
         <v>973265.08127999189</v>
       </c>
       <c r="E87" s="60">
-        <v>178.32811346650587</v>
+        <v>178.32811343084896</v>
       </c>
       <c r="F87" s="60">
-        <v>61.79</v>
+        <v>61.789499318531895</v>
       </c>
       <c r="G87" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H87" s="80" t="s">
+      <c r="H87" s="79" t="s">
         <v>110</v>
       </c>
     </row>
@@ -4162,15 +4161,15 @@
         <v>50246.946787724926</v>
       </c>
       <c r="E88" s="60">
-        <v>116.00829742715828</v>
+        <v>108.27441091036481</v>
       </c>
       <c r="F88" s="60">
-        <v>45.96</v>
+        <v>43.715100994013127</v>
       </c>
       <c r="G88" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H88" s="80" t="s">
+      <c r="H88" s="79" t="s">
         <v>110</v>
       </c>
     </row>
@@ -4185,18 +4184,18 @@
         <v>13</v>
       </c>
       <c r="D89" s="59">
-        <v>1908956.3996125823</v>
+        <v>1903069.0044591248</v>
       </c>
       <c r="E89" s="60">
-        <v>38.669432475719425</v>
+        <v>38.669432467987427</v>
       </c>
       <c r="F89" s="60">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G89" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H89" s="80" t="s">
+      <c r="H89" s="79" t="s">
         <v>110</v>
       </c>
     </row>
@@ -4214,7 +4213,7 @@
         <v>1393813.6003874179</v>
       </c>
       <c r="E90" s="60">
-        <v>38.669432475719425</v>
+        <v>38.669432467987427</v>
       </c>
       <c r="F90" s="71">
         <v>0</v>
@@ -4222,7 +4221,7 @@
       <c r="G90" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H90" s="80" t="s">
+      <c r="H90" s="79" t="s">
         <v>110</v>
       </c>
     </row>
@@ -4240,7 +4239,7 @@
         <v>413648.97193228296</v>
       </c>
       <c r="E91" s="60">
-        <v>142.28276487374458</v>
+        <v>142.28276484529499</v>
       </c>
       <c r="F91" s="71">
         <v>0</v>
@@ -4248,7 +4247,7 @@
       <c r="G91" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H91" s="80" t="s">
+      <c r="H91" s="79" t="s">
         <v>110</v>
       </c>
     </row>
@@ -4266,15 +4265,15 @@
         <v>461167</v>
       </c>
       <c r="E92" s="65">
-        <v>46.40331897086331</v>
+        <v>46.403318961584908</v>
       </c>
       <c r="F92" s="65">
-        <v>17.989999999999998</v>
+        <v>17.987644010001613</v>
       </c>
       <c r="G92" s="66" t="s">
         <v>38</v>
       </c>
-      <c r="H92" s="81" t="s">
+      <c r="H92" s="80" t="s">
         <v>110</v>
       </c>
     </row>
@@ -4302,15 +4301,15 @@
         <v>170846</v>
       </c>
       <c r="E94" s="69">
-        <v>38.669432475719425</v>
+        <v>38.669432467987427</v>
       </c>
       <c r="F94" s="69">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G94" s="70" t="s">
         <v>39</v>
       </c>
-      <c r="H94" s="79" t="s">
+      <c r="H94" s="78" t="s">
         <v>110</v>
       </c>
     </row>
@@ -4330,15 +4329,15 @@
         <v>115637</v>
       </c>
       <c r="E95" s="60">
-        <v>178.32811346650587</v>
+        <v>178.32811343084896</v>
       </c>
       <c r="F95" s="60">
-        <v>61.79</v>
+        <v>61.789499318531895</v>
       </c>
       <c r="G95" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H95" s="80" t="s">
+      <c r="H95" s="79" t="s">
         <v>110</v>
       </c>
     </row>
@@ -4358,15 +4357,15 @@
         <v>71990</v>
       </c>
       <c r="E96" s="60">
-        <v>527.6</v>
+        <v>549.96635307824874</v>
       </c>
       <c r="F96" s="60">
-        <v>76.02</v>
+        <v>70.007057148052098</v>
       </c>
       <c r="G96" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H96" s="80" t="s">
+      <c r="H96" s="79" t="s">
         <v>110</v>
       </c>
     </row>
@@ -4386,15 +4385,15 @@
         <v>973265.08127999189</v>
       </c>
       <c r="E97" s="60">
-        <v>178.32811346650587</v>
+        <v>178.32811343084896</v>
       </c>
       <c r="F97" s="60">
-        <v>61.79</v>
+        <v>61.789499318531895</v>
       </c>
       <c r="G97" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H97" s="80" t="s">
+      <c r="H97" s="79" t="s">
         <v>110</v>
       </c>
     </row>
@@ -4414,15 +4413,15 @@
         <v>50246.946787724926</v>
       </c>
       <c r="E98" s="60">
-        <v>256.89722896322456</v>
+        <v>248.09003281726135</v>
       </c>
       <c r="F98" s="60">
-        <v>45.96</v>
+        <v>45.962687596827379</v>
       </c>
       <c r="G98" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H98" s="80" t="s">
+      <c r="H98" s="79" t="s">
         <v>110</v>
       </c>
     </row>
@@ -4439,18 +4438,18 @@
         <v>Returning band 1</v>
       </c>
       <c r="D99" s="59">
-        <v>1908956.3996125823</v>
+        <v>1903069.0044591248</v>
       </c>
       <c r="E99" s="60">
-        <v>36.699604137603508</v>
+        <v>35.441433259608765</v>
       </c>
       <c r="F99" s="60">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G99" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H99" s="80" t="s">
+      <c r="H99" s="79" t="s">
         <v>110</v>
       </c>
     </row>
@@ -4470,7 +4469,7 @@
         <v>1393813.6003874179</v>
       </c>
       <c r="E100" s="60">
-        <v>36.699604137603508</v>
+        <v>35.441433259608765</v>
       </c>
       <c r="F100" s="71">
         <v>0</v>
@@ -4478,7 +4477,7 @@
       <c r="G100" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H100" s="80" t="s">
+      <c r="H100" s="79" t="s">
         <v>110</v>
       </c>
     </row>
@@ -4498,7 +4497,7 @@
         <v>413648.97193228296</v>
       </c>
       <c r="E101" s="60">
-        <v>142.28276487374458</v>
+        <v>142.28276484529499</v>
       </c>
       <c r="F101" s="71">
         <v>0</v>
@@ -4506,7 +4505,7 @@
       <c r="G101" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H101" s="80" t="s">
+      <c r="H101" s="79" t="s">
         <v>110</v>
       </c>
     </row>
@@ -4529,12 +4528,12 @@
         <v>75</v>
       </c>
       <c r="F102" s="65">
-        <v>17.989999999999998</v>
+        <v>17.987644010001613</v>
       </c>
       <c r="G102" s="50" t="s">
         <v>39</v>
       </c>
-      <c r="H102" s="81" t="s">
+      <c r="H102" s="80" t="s">
         <v>110</v>
       </c>
     </row>
@@ -4557,15 +4556,15 @@
         <v>106648</v>
       </c>
       <c r="E104" s="69">
-        <v>37.749442845846509</v>
+        <v>37.749442809183094</v>
       </c>
       <c r="F104" s="69">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G104" s="52" t="s">
         <v>38</v>
       </c>
-      <c r="H104" s="79" t="s">
+      <c r="H104" s="78" t="s">
         <v>111</v>
       </c>
     </row>
@@ -4583,15 +4582,15 @@
         <v>57472</v>
       </c>
       <c r="E105" s="60">
-        <v>181.47748086328383</v>
+        <v>181.47748068702737</v>
       </c>
       <c r="F105" s="60">
-        <v>61.79</v>
+        <v>61.789499318531895</v>
       </c>
       <c r="G105" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H105" s="80" t="s">
+      <c r="H105" s="79" t="s">
         <v>111</v>
       </c>
     </row>
@@ -4609,15 +4608,15 @@
         <v>62643</v>
       </c>
       <c r="E106" s="60">
-        <v>397.30976743385634</v>
+        <v>397.30976704797695</v>
       </c>
       <c r="F106" s="60">
-        <v>75.08</v>
+        <v>76.024503939645342</v>
       </c>
       <c r="G106" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H106" s="80" t="s">
+      <c r="H106" s="79" t="s">
         <v>111</v>
       </c>
     </row>
@@ -4635,15 +4634,15 @@
         <v>939862.23797267035</v>
       </c>
       <c r="E107" s="60">
-        <v>181.47748086328383</v>
+        <v>181.47748068702737</v>
       </c>
       <c r="F107" s="60">
-        <v>61.79</v>
+        <v>61.789499318531895</v>
       </c>
       <c r="G107" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H107" s="80" t="s">
+      <c r="H107" s="79" t="s">
         <v>111</v>
       </c>
     </row>
@@ -4661,15 +4660,15 @@
         <v>42701.133603267248</v>
       </c>
       <c r="E108" s="60">
-        <v>113.24832853753952</v>
+        <v>105.69843986571267</v>
       </c>
       <c r="F108" s="60">
-        <v>45.96</v>
+        <v>43.715100994013127</v>
       </c>
       <c r="G108" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H108" s="80" t="s">
+      <c r="H108" s="79" t="s">
         <v>111</v>
       </c>
     </row>
@@ -4684,18 +4683,18 @@
         <v>13</v>
       </c>
       <c r="D109" s="59">
-        <v>1720683.1425587691</v>
+        <v>1715658.4478799966</v>
       </c>
       <c r="E109" s="60">
-        <v>37.749442845846509</v>
+        <v>37.749442809183094</v>
       </c>
       <c r="F109" s="60">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G109" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H109" s="80" t="s">
+      <c r="H109" s="79" t="s">
         <v>111</v>
       </c>
     </row>
@@ -4713,7 +4712,7 @@
         <v>1224615.8574412311</v>
       </c>
       <c r="E110" s="60">
-        <v>37.749442845846509</v>
+        <v>37.749442809183094</v>
       </c>
       <c r="F110" s="71">
         <v>0</v>
@@ -4721,7 +4720,7 @@
       <c r="G110" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H110" s="80" t="s">
+      <c r="H110" s="79" t="s">
         <v>111</v>
       </c>
     </row>
@@ -4739,7 +4738,7 @@
         <v>376605.62842406222</v>
       </c>
       <c r="E111" s="60">
-        <v>144.79555263393681</v>
+        <v>144.79555249330693</v>
       </c>
       <c r="F111" s="71">
         <v>0</v>
@@ -4747,7 +4746,7 @@
       <c r="G111" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H111" s="80" t="s">
+      <c r="H111" s="79" t="s">
         <v>111</v>
       </c>
     </row>
@@ -4765,15 +4764,15 @@
         <v>480906</v>
       </c>
       <c r="E112" s="65">
-        <v>45.299331415015807</v>
+        <v>45.299331371019711</v>
       </c>
       <c r="F112" s="65">
-        <v>17.989999999999998</v>
+        <v>17.987644010001613</v>
       </c>
       <c r="G112" s="66" t="s">
         <v>38</v>
       </c>
-      <c r="H112" s="81" t="s">
+      <c r="H112" s="80" t="s">
         <v>111</v>
       </c>
     </row>
@@ -4801,15 +4800,15 @@
         <v>106648</v>
       </c>
       <c r="E114" s="69">
-        <v>37.749442845846509</v>
+        <v>37.749442809183094</v>
       </c>
       <c r="F114" s="69">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G114" s="70" t="s">
         <v>39</v>
       </c>
-      <c r="H114" s="79" t="s">
+      <c r="H114" s="78" t="s">
         <v>111</v>
       </c>
     </row>
@@ -4829,15 +4828,15 @@
         <v>57472</v>
       </c>
       <c r="E115" s="60">
-        <v>181.47748086328383</v>
+        <v>181.47748068702737</v>
       </c>
       <c r="F115" s="60">
-        <v>61.79</v>
+        <v>61.789499318531895</v>
       </c>
       <c r="G115" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H115" s="80" t="s">
+      <c r="H115" s="79" t="s">
         <v>111</v>
       </c>
     </row>
@@ -4857,15 +4856,15 @@
         <v>62643</v>
       </c>
       <c r="E116" s="60">
-        <v>527.6</v>
+        <v>549.96635307824874</v>
       </c>
       <c r="F116" s="60">
-        <v>76.02</v>
+        <v>70.007057148052098</v>
       </c>
       <c r="G116" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H116" s="80" t="s">
+      <c r="H116" s="79" t="s">
         <v>111</v>
       </c>
     </row>
@@ -4885,15 +4884,15 @@
         <v>939862.23797267035</v>
       </c>
       <c r="E117" s="60">
-        <v>181.47748086328383</v>
+        <v>181.47748068702737</v>
       </c>
       <c r="F117" s="60">
-        <v>61.79</v>
+        <v>61.789499318531895</v>
       </c>
       <c r="G117" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H117" s="80" t="s">
+      <c r="H117" s="79" t="s">
         <v>111</v>
       </c>
     </row>
@@ -4913,15 +4912,15 @@
         <v>42701.133603267248</v>
       </c>
       <c r="E118" s="60">
-        <v>256.89722896322456</v>
+        <v>248.09003281726135</v>
       </c>
       <c r="F118" s="60">
-        <v>45.96</v>
+        <v>45.962687596827379</v>
       </c>
       <c r="G118" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H118" s="80" t="s">
+      <c r="H118" s="79" t="s">
         <v>111</v>
       </c>
     </row>
@@ -4938,18 +4937,18 @@
         <v>Returning band 1</v>
       </c>
       <c r="D119" s="59">
-        <v>1720683.1425587691</v>
+        <v>1715658.4478799966</v>
       </c>
       <c r="E119" s="60">
-        <v>36.699604137603508</v>
+        <v>35.441433259608765</v>
       </c>
       <c r="F119" s="60">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G119" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H119" s="80" t="s">
+      <c r="H119" s="79" t="s">
         <v>111</v>
       </c>
     </row>
@@ -4969,7 +4968,7 @@
         <v>1224615.8574412311</v>
       </c>
       <c r="E120" s="60">
-        <v>36.699604137603508</v>
+        <v>35.441433259608765</v>
       </c>
       <c r="F120" s="71">
         <v>0</v>
@@ -4977,7 +4976,7 @@
       <c r="G120" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H120" s="80" t="s">
+      <c r="H120" s="79" t="s">
         <v>111</v>
       </c>
     </row>
@@ -4997,7 +4996,7 @@
         <v>376605.62842406222</v>
       </c>
       <c r="E121" s="60">
-        <v>144.79555263393681</v>
+        <v>144.79555249330693</v>
       </c>
       <c r="F121" s="71">
         <v>0</v>
@@ -5005,7 +5004,7 @@
       <c r="G121" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H121" s="80" t="s">
+      <c r="H121" s="79" t="s">
         <v>111</v>
       </c>
     </row>
@@ -5028,12 +5027,12 @@
         <v>75</v>
       </c>
       <c r="F122" s="65">
-        <v>17.989999999999998</v>
+        <v>17.987644010001613</v>
       </c>
       <c r="G122" s="50" t="s">
         <v>39</v>
       </c>
-      <c r="H122" s="81" t="s">
+      <c r="H122" s="80" t="s">
         <v>111</v>
       </c>
     </row>
@@ -5056,15 +5055,15 @@
         <v>248695</v>
       </c>
       <c r="E124" s="69">
-        <v>35.839428789649212</v>
+        <v>35.839428805227314</v>
       </c>
       <c r="F124" s="69">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G124" s="52" t="s">
         <v>38</v>
       </c>
-      <c r="H124" s="79" t="s">
+      <c r="H124" s="78" t="s">
         <v>112</v>
       </c>
     </row>
@@ -5082,15 +5081,15 @@
         <v>145992</v>
       </c>
       <c r="E125" s="60">
-        <v>176.69378435926555</v>
+        <v>176.69378443606794</v>
       </c>
       <c r="F125" s="60">
-        <v>61.79</v>
+        <v>61.789499318531895</v>
       </c>
       <c r="G125" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H125" s="80" t="s">
+      <c r="H125" s="79" t="s">
         <v>112</v>
       </c>
     </row>
@@ -5108,15 +5107,15 @@
         <v>48289</v>
       </c>
       <c r="E126" s="60">
-        <v>371.07780452258294</v>
+        <v>371.07780468387699</v>
       </c>
       <c r="F126" s="60">
-        <v>92.96</v>
+        <v>76.024503939645342</v>
       </c>
       <c r="G126" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H126" s="80" t="s">
+      <c r="H126" s="79" t="s">
         <v>112</v>
       </c>
     </row>
@@ -5134,15 +5133,15 @@
         <v>709076.2136203578</v>
       </c>
       <c r="E127" s="60">
-        <v>176.69378435926555</v>
+        <v>176.69378443606794</v>
       </c>
       <c r="F127" s="60">
-        <v>61.79</v>
+        <v>61.789499318531895</v>
       </c>
       <c r="G127" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H127" s="80" t="s">
+      <c r="H127" s="79" t="s">
         <v>112</v>
       </c>
     </row>
@@ -5160,15 +5159,15 @@
         <v>42217.047945793951</v>
       </c>
       <c r="E128" s="60">
-        <v>107.51828636894763</v>
+        <v>100.35040065463649</v>
       </c>
       <c r="F128" s="60">
-        <v>45.96</v>
+        <v>43.715100994013127</v>
       </c>
       <c r="G128" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H128" s="80" t="s">
+      <c r="H128" s="79" t="s">
         <v>112</v>
       </c>
     </row>
@@ -5183,18 +5182,18 @@
         <v>13</v>
       </c>
       <c r="D129" s="59">
-        <v>1655805.7007587738</v>
+        <v>1651535.5873984471</v>
       </c>
       <c r="E129" s="60">
-        <v>35.839428789649212</v>
+        <v>35.839428805227314</v>
       </c>
       <c r="F129" s="60">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G129" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H129" s="80" t="s">
+      <c r="H129" s="79" t="s">
         <v>112</v>
       </c>
     </row>
@@ -5212,7 +5211,7 @@
         <v>1276332.2992412264</v>
       </c>
       <c r="E130" s="60">
-        <v>35.839428789649212</v>
+        <v>35.839428805227314</v>
       </c>
       <c r="F130" s="71">
         <v>0</v>
@@ -5220,7 +5219,7 @@
       <c r="G130" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H130" s="80" t="s">
+      <c r="H130" s="79" t="s">
         <v>112</v>
       </c>
     </row>
@@ -5238,7 +5237,7 @@
         <v>322948.73843384819</v>
       </c>
       <c r="E131" s="60">
-        <v>140.97878167349916</v>
+        <v>140.97878173477756</v>
       </c>
       <c r="F131" s="71">
         <v>0</v>
@@ -5246,7 +5245,7 @@
       <c r="G131" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H131" s="80" t="s">
+      <c r="H131" s="79" t="s">
         <v>112</v>
       </c>
     </row>
@@ -5264,15 +5263,15 @@
         <v>426680</v>
       </c>
       <c r="E132" s="65">
-        <v>43.00731454757905</v>
+        <v>43.007314566272775</v>
       </c>
       <c r="F132" s="65">
-        <v>17.989999999999998</v>
+        <v>17.987644010001613</v>
       </c>
       <c r="G132" s="66" t="s">
         <v>38</v>
       </c>
-      <c r="H132" s="81" t="s">
+      <c r="H132" s="80" t="s">
         <v>112</v>
       </c>
     </row>
@@ -5300,15 +5299,15 @@
         <v>248695</v>
       </c>
       <c r="E134" s="69">
-        <v>35.839428789649212</v>
+        <v>35.839428805227314</v>
       </c>
       <c r="F134" s="69">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G134" s="70" t="s">
         <v>39</v>
       </c>
-      <c r="H134" s="79" t="s">
+      <c r="H134" s="78" t="s">
         <v>112</v>
       </c>
     </row>
@@ -5328,15 +5327,15 @@
         <v>145992</v>
       </c>
       <c r="E135" s="60">
-        <v>176.69378435926555</v>
+        <v>176.69378443606794</v>
       </c>
       <c r="F135" s="60">
-        <v>61.79</v>
+        <v>61.789499318531895</v>
       </c>
       <c r="G135" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H135" s="80" t="s">
+      <c r="H135" s="79" t="s">
         <v>112</v>
       </c>
     </row>
@@ -5356,15 +5355,15 @@
         <v>48289</v>
       </c>
       <c r="E136" s="60">
-        <v>527.6</v>
+        <v>549.96635307824874</v>
       </c>
       <c r="F136" s="60">
-        <v>76.02</v>
+        <v>70.007057148052098</v>
       </c>
       <c r="G136" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H136" s="80" t="s">
+      <c r="H136" s="79" t="s">
         <v>112</v>
       </c>
     </row>
@@ -5384,15 +5383,15 @@
         <v>709076.2136203578</v>
       </c>
       <c r="E137" s="60">
-        <v>176.69378435926555</v>
+        <v>176.69378443606794</v>
       </c>
       <c r="F137" s="60">
-        <v>61.79</v>
+        <v>61.789499318531895</v>
       </c>
       <c r="G137" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H137" s="80" t="s">
+      <c r="H137" s="79" t="s">
         <v>112</v>
       </c>
     </row>
@@ -5412,15 +5411,15 @@
         <v>42217.047945793951</v>
       </c>
       <c r="E138" s="60">
-        <v>256.89722896322456</v>
+        <v>248.09003281726135</v>
       </c>
       <c r="F138" s="60">
-        <v>45.96</v>
+        <v>45.962687596827379</v>
       </c>
       <c r="G138" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H138" s="80" t="s">
+      <c r="H138" s="79" t="s">
         <v>112</v>
       </c>
     </row>
@@ -5437,18 +5436,18 @@
         <v>Returning band 1</v>
       </c>
       <c r="D139" s="59">
-        <v>1655805.7007587738</v>
+        <v>1651535.5873984471</v>
       </c>
       <c r="E139" s="60">
-        <v>36.699604137603508</v>
+        <v>35.441433259608765</v>
       </c>
       <c r="F139" s="60">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G139" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H139" s="80" t="s">
+      <c r="H139" s="79" t="s">
         <v>112</v>
       </c>
     </row>
@@ -5468,7 +5467,7 @@
         <v>1276332.2992412264</v>
       </c>
       <c r="E140" s="60">
-        <v>36.699604137603508</v>
+        <v>35.441433259608765</v>
       </c>
       <c r="F140" s="71">
         <v>0</v>
@@ -5476,7 +5475,7 @@
       <c r="G140" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H140" s="80" t="s">
+      <c r="H140" s="79" t="s">
         <v>112</v>
       </c>
     </row>
@@ -5496,7 +5495,7 @@
         <v>322948.73843384819</v>
       </c>
       <c r="E141" s="60">
-        <v>140.97878167349916</v>
+        <v>140.97878173477756</v>
       </c>
       <c r="F141" s="71">
         <v>0</v>
@@ -5504,7 +5503,7 @@
       <c r="G141" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H141" s="80" t="s">
+      <c r="H141" s="79" t="s">
         <v>112</v>
       </c>
     </row>
@@ -5527,12 +5526,12 @@
         <v>75</v>
       </c>
       <c r="F142" s="65">
-        <v>17.989999999999998</v>
+        <v>17.987644010001613</v>
       </c>
       <c r="G142" s="50" t="s">
         <v>39</v>
       </c>
-      <c r="H142" s="81" t="s">
+      <c r="H142" s="80" t="s">
         <v>112</v>
       </c>
     </row>
@@ -5555,15 +5554,15 @@
         <v>100295</v>
       </c>
       <c r="E144" s="69">
-        <v>36.356464595445232</v>
+        <v>36.356464583335409</v>
       </c>
       <c r="F144" s="69">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G144" s="52" t="s">
         <v>38</v>
       </c>
-      <c r="H144" s="79" t="s">
+      <c r="H144" s="78" t="s">
         <v>113</v>
       </c>
     </row>
@@ -5581,15 +5580,15 @@
         <v>61668</v>
       </c>
       <c r="E145" s="60">
-        <v>169.20371166638463</v>
+        <v>169.20371161002527</v>
       </c>
       <c r="F145" s="60">
-        <v>61.79</v>
+        <v>61.789499318531895</v>
       </c>
       <c r="G145" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H145" s="80" t="s">
+      <c r="H145" s="79" t="s">
         <v>113</v>
       </c>
     </row>
@@ -5607,15 +5606,15 @@
         <v>27518</v>
       </c>
       <c r="E146" s="60">
-        <v>364.62291792701348</v>
+        <v>364.62291780556274</v>
       </c>
       <c r="F146" s="60">
-        <v>87.68</v>
+        <v>76.024503939645342</v>
       </c>
       <c r="G146" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H146" s="80" t="s">
+      <c r="H146" s="79" t="s">
         <v>113</v>
       </c>
     </row>
@@ -5633,15 +5632,15 @@
         <v>382812.97444371646</v>
       </c>
       <c r="E147" s="60">
-        <v>169.20371166638463</v>
+        <v>169.20371161002527</v>
       </c>
       <c r="F147" s="60">
-        <v>61.79</v>
+        <v>61.789499318531895</v>
       </c>
       <c r="G147" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H147" s="80" t="s">
+      <c r="H147" s="79" t="s">
         <v>113</v>
       </c>
     </row>
@@ -5659,15 +5658,15 @@
         <v>23229.204654273493</v>
       </c>
       <c r="E148" s="60">
-        <v>109.0693937863357</v>
+        <v>101.79810083333915</v>
       </c>
       <c r="F148" s="60">
-        <v>45.96</v>
+        <v>43.715100994013127</v>
       </c>
       <c r="G148" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H148" s="80" t="s">
+      <c r="H148" s="79" t="s">
         <v>113</v>
       </c>
     </row>
@@ -5682,18 +5681,18 @@
         <v>13</v>
       </c>
       <c r="D149" s="59">
-        <v>914352.42805637419</v>
+        <v>910130.72326179477</v>
       </c>
       <c r="E149" s="60">
-        <v>36.356464595445232</v>
+        <v>36.356464583335409</v>
       </c>
       <c r="F149" s="60">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G149" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H149" s="80" t="s">
+      <c r="H149" s="79" t="s">
         <v>113</v>
       </c>
     </row>
@@ -5711,7 +5710,7 @@
         <v>679982.57194362592</v>
       </c>
       <c r="E150" s="60">
-        <v>36.356464595445232</v>
+        <v>36.356464583335409</v>
       </c>
       <c r="F150" s="71">
         <v>0</v>
@@ -5719,7 +5718,7 @@
       <c r="G150" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H150" s="80" t="s">
+      <c r="H150" s="79" t="s">
         <v>113</v>
       </c>
     </row>
@@ -5737,7 +5736,7 @@
         <v>169138.82090200999</v>
       </c>
       <c r="E151" s="60">
-        <v>135.00267262859191</v>
+        <v>135.00267258362445</v>
       </c>
       <c r="F151" s="71">
         <v>0</v>
@@ -5745,7 +5744,7 @@
       <c r="G151" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H151" s="80" t="s">
+      <c r="H151" s="79" t="s">
         <v>113</v>
       </c>
     </row>
@@ -5763,15 +5762,15 @@
         <v>208822</v>
       </c>
       <c r="E152" s="65">
-        <v>43.627757514534274</v>
+        <v>43.627757500002488</v>
       </c>
       <c r="F152" s="65">
-        <v>17.989999999999998</v>
+        <v>17.987644010001613</v>
       </c>
       <c r="G152" s="66" t="s">
         <v>38</v>
       </c>
-      <c r="H152" s="81" t="s">
+      <c r="H152" s="80" t="s">
         <v>113</v>
       </c>
     </row>
@@ -5799,15 +5798,15 @@
         <v>100295</v>
       </c>
       <c r="E154" s="69">
-        <v>36.356464595445232</v>
+        <v>36.356464583335409</v>
       </c>
       <c r="F154" s="69">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G154" s="70" t="s">
         <v>39</v>
       </c>
-      <c r="H154" s="79" t="s">
+      <c r="H154" s="78" t="s">
         <v>113</v>
       </c>
     </row>
@@ -5827,15 +5826,15 @@
         <v>61668</v>
       </c>
       <c r="E155" s="60">
-        <v>169.20371166638463</v>
+        <v>169.20371161002527</v>
       </c>
       <c r="F155" s="60">
-        <v>61.79</v>
+        <v>61.789499318531895</v>
       </c>
       <c r="G155" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H155" s="80" t="s">
+      <c r="H155" s="79" t="s">
         <v>113</v>
       </c>
     </row>
@@ -5855,15 +5854,15 @@
         <v>27518</v>
       </c>
       <c r="E156" s="60">
-        <v>527.6</v>
+        <v>549.96635307824874</v>
       </c>
       <c r="F156" s="60">
-        <v>76.02</v>
+        <v>70.007057148052098</v>
       </c>
       <c r="G156" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H156" s="80" t="s">
+      <c r="H156" s="79" t="s">
         <v>113</v>
       </c>
     </row>
@@ -5883,15 +5882,15 @@
         <v>382812.97444371646</v>
       </c>
       <c r="E157" s="60">
-        <v>169.20371166638463</v>
+        <v>169.20371161002527</v>
       </c>
       <c r="F157" s="60">
-        <v>61.79</v>
+        <v>61.789499318531895</v>
       </c>
       <c r="G157" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H157" s="80" t="s">
+      <c r="H157" s="79" t="s">
         <v>113</v>
       </c>
     </row>
@@ -5911,15 +5910,15 @@
         <v>23229.204654273493</v>
       </c>
       <c r="E158" s="60">
-        <v>256.89722896322456</v>
+        <v>248.09003281726135</v>
       </c>
       <c r="F158" s="60">
-        <v>45.96</v>
+        <v>45.962687596827379</v>
       </c>
       <c r="G158" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H158" s="80" t="s">
+      <c r="H158" s="79" t="s">
         <v>113</v>
       </c>
     </row>
@@ -5936,18 +5935,18 @@
         <v>Returning band 1</v>
       </c>
       <c r="D159" s="59">
-        <v>914352.42805637419</v>
+        <v>910130.72326179477</v>
       </c>
       <c r="E159" s="60">
-        <v>36.699604137603508</v>
+        <v>35.441433259608765</v>
       </c>
       <c r="F159" s="60">
-        <v>23.49</v>
+        <v>23.486821568684874</v>
       </c>
       <c r="G159" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H159" s="80" t="s">
+      <c r="H159" s="79" t="s">
         <v>113</v>
       </c>
     </row>
@@ -5967,7 +5966,7 @@
         <v>679982.57194362592</v>
       </c>
       <c r="E160" s="60">
-        <v>36.699604137603508</v>
+        <v>35.441433259608765</v>
       </c>
       <c r="F160" s="71">
         <v>0</v>
@@ -5975,7 +5974,7 @@
       <c r="G160" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H160" s="80" t="s">
+      <c r="H160" s="79" t="s">
         <v>113</v>
       </c>
     </row>
@@ -5995,7 +5994,7 @@
         <v>169138.82090200999</v>
       </c>
       <c r="E161" s="60">
-        <v>135.00267262859191</v>
+        <v>135.00267258362445</v>
       </c>
       <c r="F161" s="71">
         <v>0</v>
@@ -6003,7 +6002,7 @@
       <c r="G161" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H161" s="80" t="s">
+      <c r="H161" s="79" t="s">
         <v>113</v>
       </c>
     </row>
@@ -6026,12 +6025,12 @@
         <v>75</v>
       </c>
       <c r="F162" s="65">
-        <v>17.989999999999998</v>
+        <v>17.987644010001613</v>
       </c>
       <c r="G162" s="50" t="s">
         <v>39</v>
       </c>
-      <c r="H162" s="81" t="s">
+      <c r="H162" s="80" t="s">
         <v>113</v>
       </c>
     </row>

</xml_diff>